<commit_message>
Refactor charts layout and update styles; change chart type to bar and improve scrollbar design
</commit_message>
<xml_diff>
--- a/texts/tablici/grafiki_diplomna.xlsx
+++ b/texts/tablici/grafiki_diplomna.xlsx
@@ -31,7 +31,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId12" roundtripDataChecksum="lgenbz6NjUnzMUioi7paK7LQCPDBvcC7ZBdaiIs7JGk="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId12" roundtripDataChecksum="KpWV8/yAHGskgR790muf+f/lYacE0feDjEJjn882Ilc="/>
     </ext>
   </extLst>
 </workbook>
@@ -461,11 +461,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1476221005"/>
-        <c:axId val="1985324977"/>
+        <c:axId val="1811820974"/>
+        <c:axId val="1626221368"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1476221005"/>
+        <c:axId val="1811820974"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -517,10 +517,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1985324977"/>
+        <c:crossAx val="1626221368"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1985324977"/>
+        <c:axId val="1626221368"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -584,7 +584,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1476221005"/>
+        <c:crossAx val="1811820974"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -645,11 +645,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1237142645"/>
-        <c:axId val="508997159"/>
+        <c:axId val="745147028"/>
+        <c:axId val="61143969"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1237142645"/>
+        <c:axId val="745147028"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -701,10 +701,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="508997159"/>
+        <c:crossAx val="61143969"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="508997159"/>
+        <c:axId val="61143969"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -768,7 +768,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1237142645"/>
+        <c:crossAx val="745147028"/>
         <c:crosses val="max"/>
       </c:valAx>
     </c:plotArea>
@@ -872,11 +872,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1768076660"/>
-        <c:axId val="1606690474"/>
+        <c:axId val="2034887808"/>
+        <c:axId val="1827559814"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1768076660"/>
+        <c:axId val="2034887808"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -928,10 +928,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1606690474"/>
+        <c:crossAx val="1827559814"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1606690474"/>
+        <c:axId val="1827559814"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1006,7 +1006,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1768076660"/>
+        <c:crossAx val="2034887808"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1097,11 +1097,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1268500209"/>
-        <c:axId val="1979643143"/>
+        <c:axId val="722121506"/>
+        <c:axId val="1820262685"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1268500209"/>
+        <c:axId val="722121506"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1153,10 +1153,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1979643143"/>
+        <c:crossAx val="1820262685"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1979643143"/>
+        <c:axId val="1820262685"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1231,7 +1231,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1268500209"/>
+        <c:crossAx val="722121506"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1587,11 +1587,11 @@
             </c:numLit>
           </c:bubbleSize>
         </c:ser>
-        <c:axId val="854181637"/>
-        <c:axId val="1950077553"/>
+        <c:axId val="920782204"/>
+        <c:axId val="1884514100"/>
       </c:bubbleChart>
       <c:valAx>
-        <c:axId val="854181637"/>
+        <c:axId val="920782204"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1666,10 +1666,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1950077553"/>
+        <c:crossAx val="1884514100"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1950077553"/>
+        <c:axId val="1884514100"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1744,7 +1744,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="854181637"/>
+        <c:crossAx val="920782204"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1924,7 +1924,7 @@
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
               </a:rPr>
-              <a:t>Многокритериално търсене</a:t>
+              <a:t>USB Flash, SSD, HDD, SD карта and CD/DVD</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1932,18 +1932,9 @@
       <c:overlay val="0"/>
     </c:title>
     <c:plotArea>
-      <c:layout>
-        <c:manualLayout>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="0.18091666666666664"/>
-          <c:y val="0.2574123989218329"/>
-          <c:w val="0.6449166666666667"/>
-          <c:h val="0.6925876010781667"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:radarChart>
-        <c:radarStyle val="marker"/>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -1953,15 +1944,15 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln cmpd="sng" w="19050">
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln cmpd="sng">
               <a:solidFill>
-                <a:srgbClr val="4F81BD"/>
+                <a:srgbClr val="000000"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
           <c:cat>
             <c:strRef>
               <c:f>'Многокритериално сравнение'!$A$2:$A$7</c:f>
@@ -1973,7 +1964,6 @@
               <c:numCache/>
             </c:numRef>
           </c:val>
-          <c:smooth val="1"/>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -1984,15 +1974,15 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln cmpd="sng" w="19050">
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln cmpd="sng">
               <a:solidFill>
-                <a:srgbClr val="C0504D"/>
+                <a:srgbClr val="000000"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
           <c:cat>
             <c:strRef>
               <c:f>'Многокритериално сравнение'!$A$2:$A$7</c:f>
@@ -2004,7 +1994,6 @@
               <c:numCache/>
             </c:numRef>
           </c:val>
-          <c:smooth val="1"/>
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
@@ -2015,15 +2004,15 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln cmpd="sng" w="19050">
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln cmpd="sng">
               <a:solidFill>
-                <a:srgbClr val="9BBB59"/>
+                <a:srgbClr val="000000"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
           <c:cat>
             <c:strRef>
               <c:f>'Многокритериално сравнение'!$A$2:$A$7</c:f>
@@ -2035,7 +2024,6 @@
               <c:numCache/>
             </c:numRef>
           </c:val>
-          <c:smooth val="1"/>
         </c:ser>
         <c:ser>
           <c:idx val="3"/>
@@ -2046,15 +2034,15 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln cmpd="sng" w="19050">
+            <a:solidFill>
+              <a:schemeClr val="accent4"/>
+            </a:solidFill>
+            <a:ln cmpd="sng">
               <a:solidFill>
-                <a:srgbClr val="8064A2"/>
+                <a:srgbClr val="000000"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
           <c:cat>
             <c:strRef>
               <c:f>'Многокритериално сравнение'!$A$2:$A$7</c:f>
@@ -2066,7 +2054,6 @@
               <c:numCache/>
             </c:numRef>
           </c:val>
-          <c:smooth val="1"/>
         </c:ser>
         <c:ser>
           <c:idx val="4"/>
@@ -2077,15 +2064,15 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln cmpd="sng" w="19050">
+            <a:solidFill>
+              <a:schemeClr val="accent5"/>
+            </a:solidFill>
+            <a:ln cmpd="sng">
               <a:solidFill>
-                <a:srgbClr val="4BACC6"/>
+                <a:srgbClr val="000000"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
           <c:cat>
             <c:strRef>
               <c:f>'Многокритериално сравнение'!$A$2:$A$7</c:f>
@@ -2097,18 +2084,17 @@
               <c:numCache/>
             </c:numRef>
           </c:val>
-          <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="1561732390"/>
-        <c:axId val="878043539"/>
-      </c:radarChart>
+        <c:axId val="1212684794"/>
+        <c:axId val="1094705299"/>
+      </c:barChart>
       <c:catAx>
-        <c:axId val="1561732390"/>
+        <c:axId val="1212684794"/>
         <c:scaling>
-          <c:orientation val="minMax"/>
+          <c:orientation val="maxMin"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="b"/>
+        <c:axPos val="l"/>
         <c:title>
           <c:tx>
             <c:rich>
@@ -2130,7 +2116,7 @@
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
                   </a:rPr>
-                  <a:t/>
+                  <a:t>Column 1</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -2155,15 +2141,15 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="878043539"/>
+        <c:crossAx val="1094705299"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="878043539"/>
+        <c:axId val="1094705299"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="l"/>
+        <c:axPos val="b"/>
         <c:majorGridlines>
           <c:spPr>
             <a:ln>
@@ -2233,7 +2219,8 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1561732390"/>
+        <c:crossAx val="1212684794"/>
+        <c:crosses val="max"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2324,11 +2311,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="347888837"/>
-        <c:axId val="1917946510"/>
+        <c:axId val="1759487066"/>
+        <c:axId val="1495673211"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="347888837"/>
+        <c:axId val="1759487066"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2380,10 +2367,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1917946510"/>
+        <c:crossAx val="1495673211"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1917946510"/>
+        <c:axId val="1495673211"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2458,7 +2445,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="347888837"/>
+        <c:crossAx val="1759487066"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2669,14 +2656,14 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>19050</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="5857875" cy="3448050"/>
+    <xdr:ext cx="5715000" cy="6010275"/>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="710207037" name="Chart 7" title="Chart"/>
+        <xdr:cNvPr id="1969329875" name="Chart 7" title="Chart"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>

</xml_diff>